<commit_message>
Version Final de Race Detector
</commit_message>
<xml_diff>
--- a/participantes.xlsx
+++ b/participantes.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,32 +39,11 @@
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-    </font>
-    <font>
       <b val="1"/>
       <color rgb="00006100"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -75,24 +54,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF4472C4"/>
         <bgColor rgb="FF4472C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -120,19 +81,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -498,19 +453,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="7"/>
+    <col width="15.109375" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="30.33203125" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="13.44140625" customWidth="1" min="8" max="8"/>
+    <col width="12.5546875" customWidth="1" min="9" max="9"/>
+    <col width="16.6640625" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.6" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cédula</t>
+          <t>Cedula</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -525,22 +485,37 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Dirección</t>
+          <t>Edad</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Distancia</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Contacto</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Dorsal</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Estado Pago</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Número Dorsal</t>
         </is>
       </c>
     </row>
@@ -590,7 +565,59 @@
           <t>100</t>
         </is>
       </c>
-      <c r="J2" s="9" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>PAGADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1802</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Manuel</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Ramirez</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>20K</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>manuel@gmail.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1212</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>JUVENIL</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>205</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>PAGADO</t>
         </is>

</xml_diff>